<commit_message>
Valida Fase 5: corrige fórmula P7 no formulário e adiciona testes de scores e filtros
</commit_message>
<xml_diff>
--- a/formulario/F_O_025_Formulario_Maturidade_Planos.xlsx
+++ b/formulario/F_O_025_Formulario_Maturidade_Planos.xlsx
@@ -2242,8 +2242,8 @@
         <v>-1</v>
       </c>
       <c r="P7" s="4">
-        <f>IF(COUNTA(G7,H7,J7)=0,"",ROUND(AVERAGE(L7:N7)*100,0))</f>
-        <v>100</v>
+        <f>IF(COUNTA(G7,H7,J7,K7)=0,"",ROUND(AVERAGE(L7:O7)*100,0))</f>
+        <v>50</v>
       </c>
       <c r="Q7" s="6">
         <f t="shared" si="4"/>

</xml_diff>